<commit_message>
feat: complete Categories 8-14 generation, persistence, and backups (202 services)
</commit_message>
<xml_diff>
--- a/backend/backups/category8_education_coaching_FINAL.xlsx
+++ b/backend/backups/category8_education_coaching_FINAL.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -507,12 +507,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d9cc76c1-de06-5737-8945-30bb558d5a13</t>
+          <t>7c32be20-c182-520a-81aa-023010c92589</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 1</t>
+          <t>Competitive Exam Coaching Service Variation 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -522,11 +522,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>950</v>
+        <v>650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -535,34 +535,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.023255+00:00</t>
+          <t>2026-09-05T15:22:47.062385+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.023255+00:00</t>
+          <t>2026-09-05T15:40:26.038841+00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>293ae0d9-5f80-5635-93cb-459e7ffcb6c1</t>
+          <t>68a89425-9371-557a-9350-1ab2b72dc715</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 2</t>
+          <t>Competitive Exam Coaching Service Variation 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -572,11 +572,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -585,34 +585,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.028305+00:00</t>
+          <t>2026-09-05T15:22:47.064979+00:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.028305+00:00</t>
+          <t>2026-09-05T15:40:26.043639+00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>946f1a7c-5278-5372-9aee-571229c7d7a7</t>
+          <t>b4401132-f924-51fd-9ae0-7c765ac1c0d8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 3</t>
+          <t>Competitive Exam Coaching Service Variation 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -622,11 +622,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1250</v>
+        <v>950</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -635,34 +635,34 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.031218+00:00</t>
+          <t>2026-09-05T15:22:47.067888+00:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.031218+00:00</t>
+          <t>2026-09-05T15:40:26.047171+00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bf24b529-26a3-56e7-ba4f-85893181cd5d</t>
+          <t>c48b2fba-232c-52f6-8502-e4569b397a26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 4</t>
+          <t>Competitive Exam Coaching Service Variation 4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -672,11 +672,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1400</v>
+        <v>1100</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -685,34 +685,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.035452+00:00</t>
+          <t>2026-09-05T15:22:47.070369+00:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.035452+00:00</t>
+          <t>2026-09-05T15:40:26.050213+00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e3a74561-e859-5f36-ab07-545c6823fbd1</t>
+          <t>e35ee0c0-dce3-52f3-9e81-29c86c1ffd37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 5</t>
+          <t>Competitive Exam Coaching Service Variation 5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -722,11 +722,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1550</v>
+        <v>1250</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -735,34 +735,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.039114+00:00</t>
+          <t>2026-09-05T15:22:47.072557+00:00</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.039114+00:00</t>
+          <t>2026-09-05T15:40:26.053354+00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>c9b53453-8a57-5ae6-843c-15688915434b</t>
+          <t>de519db1-8c08-5b9e-877e-fa214ff39a55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 6</t>
+          <t>Competitive Exam Coaching Service Variation 6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -772,11 +772,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -785,34 +785,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.041425+00:00</t>
+          <t>2026-09-05T15:22:47.074889+00:00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.041425+00:00</t>
+          <t>2026-09-05T15:40:26.055776+00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>d62dfd9c-d29f-576c-9470-2bbae0544e3a</t>
+          <t>4bf49dce-f45c-55e3-a14e-1f185bda38ac</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Academic Tutoring Service Variation 7</t>
+          <t>Competitive Exam Coaching Service Variation 7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -822,11 +822,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Academic Tutoring</t>
+          <t>Competitive Exam Coaching</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1850</v>
+        <v>1550</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -835,34 +835,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[{"text": "Expert academic tutoring tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Academic Tutoring Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional competitive exam coaching coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Competitive Exam Coaching instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.044343+00:00</t>
+          <t>2026-09-05T15:40:26.057957+00:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.044343+00:00</t>
+          <t>2026-09-05T15:40:26.057957+00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6cdfea65-f777-5015-ab14-9629e747eb08</t>
+          <t>63f30e5d-4fa8-5c19-946f-1a524b8b74c1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 1</t>
+          <t>Language Coaching Service Variation 6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>950</v>
+        <v>1700</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -895,24 +895,24 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.046691+00:00</t>
+          <t>2026-09-05T15:22:47.059934+00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.046691+00:00</t>
+          <t>2026-09-05T15:22:47.059934+00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>41f10521-548d-5a2d-a4a9-840503b42220</t>
+          <t>f1106c8b-997a-5d06-a1b6-b30fd8b10523</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 2</t>
+          <t>Language &amp; Communication Service Variation 1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -922,11 +922,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -935,34 +935,34 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.049835+00:00</t>
+          <t>2026-09-05T15:22:47.089751+00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.049835+00:00</t>
+          <t>2026-09-05T15:40:26.060681+00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3c7771ad-a2b2-51ce-8846-bbe481a7c7c1</t>
+          <t>d11d4e8e-10ab-52fa-8b31-c974ba7f8906</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 3</t>
+          <t>Language &amp; Communication Service Variation 2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -972,11 +972,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1250</v>
+        <v>800</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -985,34 +985,34 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.052666+00:00</t>
+          <t>2026-09-05T15:22:47.092066+00:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.052666+00:00</t>
+          <t>2026-09-05T15:40:26.063121+00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>453266d6-b237-5e06-8df4-33eda2c614ee</t>
+          <t>245d6207-15de-5adc-9b1b-7c387c372955</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 4</t>
+          <t>Language &amp; Communication Service Variation 3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1022,11 +1022,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1400</v>
+        <v>950</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1035,34 +1035,34 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.055059+00:00</t>
+          <t>2026-09-05T15:22:47.094264+00:00</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.055059+00:00</t>
+          <t>2026-09-05T15:40:26.065533+00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>479f80e0-44a1-531c-9ad2-ade93e865775</t>
+          <t>e4f0a121-e2bb-5118-a516-7a3c16944184</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 5</t>
+          <t>Language &amp; Communication Service Variation 4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1072,11 +1072,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1550</v>
+        <v>1100</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1085,34 +1085,34 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.057378+00:00</t>
+          <t>2026-09-05T15:22:47.096490+00:00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.057378+00:00</t>
+          <t>2026-09-05T15:40:26.068388+00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>63f30e5d-4fa8-5c19-946f-1a524b8b74c1</t>
+          <t>a05334fd-3b60-510c-ae8c-8d53275a302e</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 6</t>
+          <t>Language &amp; Communication Service Variation 5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1122,11 +1122,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1700</v>
+        <v>1250</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1135,34 +1135,34 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.059934+00:00</t>
+          <t>2026-09-05T15:22:47.098887+00:00</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.059934+00:00</t>
+          <t>2026-09-05T15:40:26.070890+00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7c32be20-c182-520a-81aa-023010c92589</t>
+          <t>6cdfea65-f777-5015-ab14-9629e747eb08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 1</t>
+          <t>Music &amp; Arts Lessons Service Variation 1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1172,11 +1172,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>950</v>
+        <v>650</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1185,34 +1185,34 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.062385+00:00</t>
+          <t>2026-09-05T15:22:47.046691+00:00</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.062385+00:00</t>
+          <t>2026-09-05T15:40:26.073488+00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>68a89425-9371-557a-9350-1ab2b72dc715</t>
+          <t>41f10521-548d-5a2d-a4a9-840503b42220</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 2</t>
+          <t>Music &amp; Arts Lessons Service Variation 2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1222,11 +1222,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1235,34 +1235,34 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.064979+00:00</t>
+          <t>2026-09-05T15:22:47.049835+00:00</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.064979+00:00</t>
+          <t>2026-09-05T15:40:26.076124+00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>b4401132-f924-51fd-9ae0-7c765ac1c0d8</t>
+          <t>3c7771ad-a2b2-51ce-8846-bbe481a7c7c1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 3</t>
+          <t>Music &amp; Arts Lessons Service Variation 3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1250</v>
+        <v>950</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1285,34 +1285,34 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.067888+00:00</t>
+          <t>2026-09-05T15:22:47.052666+00:00</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.067888+00:00</t>
+          <t>2026-09-05T15:40:26.078483+00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>c48b2fba-232c-52f6-8502-e4569b397a26</t>
+          <t>453266d6-b237-5e06-8df4-33eda2c614ee</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 4</t>
+          <t>Music &amp; Arts Lessons Service Variation 4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1400</v>
+        <v>1100</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1335,34 +1335,34 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.070369+00:00</t>
+          <t>2026-09-05T15:22:47.055059+00:00</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.070369+00:00</t>
+          <t>2026-09-05T15:40:26.081162+00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>e35ee0c0-dce3-52f3-9e81-29c86c1ffd37</t>
+          <t>479f80e0-44a1-531c-9ad2-ade93e865775</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 5</t>
+          <t>Music &amp; Arts Lessons Service Variation 5</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1372,11 +1372,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1550</v>
+        <v>1250</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1385,34 +1385,34 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.072557+00:00</t>
+          <t>2026-09-05T15:22:47.057378+00:00</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.072557+00:00</t>
+          <t>2026-09-05T15:40:26.083919+00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>de519db1-8c08-5b9e-877e-fa214ff39a55</t>
+          <t>d9cc76c1-de06-5737-8945-30bb558d5a13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Service Variation 6</t>
+          <t>School Tutoring (K-12) Service Variation 1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1422,11 +1422,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Music &amp; Arts</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1700</v>
+        <v>650</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1435,34 +1435,34 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>[{"text": "Expert music &amp; arts tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Music &amp; Arts Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.074889+00:00</t>
+          <t>2026-09-05T15:22:47.023255+00:00</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.074889+00:00</t>
+          <t>2026-09-05T15:40:26.087401+00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>b3caa66a-909e-5c9b-8e28-066ea5298ca7</t>
+          <t>293ae0d9-5f80-5635-93cb-459e7ffcb6c1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching Service Variation 1</t>
+          <t>School Tutoring (K-12) Service Variation 2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1472,11 +1472,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>950</v>
+        <v>800</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1485,34 +1485,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>[{"text": "Expert sports &amp; fitness coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Sports &amp; Fitness Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.077035+00:00</t>
+          <t>2026-09-05T15:22:47.028305+00:00</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.077035+00:00</t>
+          <t>2026-09-05T15:40:26.089859+00:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3a2c9ca8-d9fb-5031-b211-e6031179640d</t>
+          <t>946f1a7c-5278-5372-9aee-571229c7d7a7</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching Service Variation 2</t>
+          <t>School Tutoring (K-12) Service Variation 3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1522,11 +1522,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1100</v>
+        <v>950</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1535,34 +1535,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>[{"text": "Expert sports &amp; fitness coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Sports &amp; Fitness Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.079289+00:00</t>
+          <t>2026-09-05T15:22:47.031218+00:00</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.079289+00:00</t>
+          <t>2026-09-05T15:40:26.092758+00:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fd8b9cf7-cd66-5e92-9e64-185217363d64</t>
+          <t>bf24b529-26a3-56e7-ba4f-85893181cd5d</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching Service Variation 3</t>
+          <t>School Tutoring (K-12) Service Variation 4</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1572,11 +1572,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1250</v>
+        <v>1100</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1585,34 +1585,34 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>[{"text": "Expert sports &amp; fitness coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Sports &amp; Fitness Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.082206+00:00</t>
+          <t>2026-09-05T15:22:47.035452+00:00</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.082206+00:00</t>
+          <t>2026-09-05T15:40:26.095081+00:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>df4be4ea-2f76-566a-8ad7-db35cbbfafb0</t>
+          <t>e3a74561-e859-5f36-ab07-545c6823fbd1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching Service Variation 4</t>
+          <t>School Tutoring (K-12) Service Variation 5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1400</v>
+        <v>1250</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1635,34 +1635,34 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>[{"text": "Expert sports &amp; fitness coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Sports &amp; Fitness Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.085005+00:00</t>
+          <t>2026-09-05T15:22:47.039114+00:00</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.085005+00:00</t>
+          <t>2026-09-05T15:40:26.098037+00:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>22edd7f9-7d44-5119-aacc-7979474a88f5</t>
+          <t>c9b53453-8a57-5ae6-843c-15688915434b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching Service Variation 5</t>
+          <t>School Tutoring (K-12) Service Variation 6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1672,11 +1672,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sports &amp; Fitness Coaching</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1550</v>
+        <v>1400</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1685,34 +1685,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>[{"text": "Expert sports &amp; fitness coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Sports &amp; Fitness Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.087244+00:00</t>
+          <t>2026-09-05T15:22:47.041425+00:00</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.087244+00:00</t>
+          <t>2026-09-05T15:40:26.101192+00:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>f1106c8b-997a-5d06-a1b6-b30fd8b10523</t>
+          <t>d62dfd9c-d29f-576c-9470-2bbae0544e3a</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Test Preparation Service Variation 1</t>
+          <t>School Tutoring (K-12) Service Variation 7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1722,11 +1722,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Test Preparation</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>950</v>
+        <v>1550</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1735,34 +1735,34 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.089751+00:00</t>
+          <t>2026-09-05T15:22:47.044343+00:00</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.089751+00:00</t>
+          <t>2026-09-05T15:40:26.103546+00:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>d11d4e8e-10ab-52fa-8b31-c974ba7f8906</t>
+          <t>b3caa66a-909e-5c9b-8e28-066ea5298ca7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Test Preparation Service Variation 2</t>
+          <t>Skills &amp; Hobby Classes Service Variation 1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Test Preparation</t>
+          <t>Skills &amp; Hobby Classes</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1785,34 +1785,34 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.092066+00:00</t>
+          <t>2026-09-05T15:22:47.077035+00:00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.092066+00:00</t>
+          <t>2026-09-05T15:40:26.105860+00:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>245d6207-15de-5adc-9b1b-7c387c372955</t>
+          <t>3a2c9ca8-d9fb-5031-b211-e6031179640d</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Test Preparation Service Variation 3</t>
+          <t>Skills &amp; Hobby Classes Service Variation 2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1822,11 +1822,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Test Preparation</t>
+          <t>Skills &amp; Hobby Classes</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1250</v>
+        <v>800</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1835,34 +1835,34 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.094264+00:00</t>
+          <t>2026-09-05T15:22:47.079289+00:00</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.094264+00:00</t>
+          <t>2026-09-05T15:40:26.108502+00:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>e4f0a121-e2bb-5118-a516-7a3c16944184</t>
+          <t>fd8b9cf7-cd66-5e92-9e64-185217363d64</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Test Preparation Service Variation 4</t>
+          <t>Skills &amp; Hobby Classes Service Variation 3</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1872,11 +1872,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Test Preparation</t>
+          <t>Skills &amp; Hobby Classes</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1400</v>
+        <v>950</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1885,34 +1885,34 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.096490+00:00</t>
+          <t>2026-09-05T15:22:47.082206+00:00</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.096490+00:00</t>
+          <t>2026-09-05T15:40:26.110846+00:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>a05334fd-3b60-510c-ae8c-8d53275a302e</t>
+          <t>df4be4ea-2f76-566a-8ad7-db35cbbfafb0</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Test Preparation Service Variation 5</t>
+          <t>Skills &amp; Hobby Classes Service Variation 4</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1922,11 +1922,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Test Preparation</t>
+          <t>Skills &amp; Hobby Classes</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1550</v>
+        <v>1100</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1935,70 +1935,170 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.098887+00:00</t>
+          <t>2026-09-05T15:22:47.085005+00:00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.098887+00:00</t>
+          <t>2026-09-05T15:40:26.114213+00:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>22edd7f9-7d44-5119-aacc-7979474a88f5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Skills &amp; Hobby Classes Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>8. Education, Teachers &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Skills &amp; Hobby Classes</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:22:47.087244+00:00</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:40:26.117877+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>f1093f34-1774-5635-ad64-bb37eb928fb5</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Skills &amp; Hobby Classes Service Variation 6</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8. Education, Teachers &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Skills &amp; Hobby Classes</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:40:26.120455+00:00</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:40:26.120455+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>1b791937-c35c-5f48-83c8-e2f133823421</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Test Preparation Service Variation 6</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>8. Education, Teachers &amp; Coaching</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>8. Education, Teachers &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>Test Preparation</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E33" t="n">
         <v>1700</v>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>2026-09-05T15:22:47.101322+00:00</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>2026-09-05T15:22:47.101322+00:00</t>
         </is>

</xml_diff>

<commit_message>
fix: remove 2 stale Cat 8 stubs, correct total to 457 services (DB verified)
</commit_message>
<xml_diff>
--- a/backend/backups/category8_education_coaching_FINAL.xlsx
+++ b/backend/backups/category8_education_coaching_FINAL.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -857,12 +857,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>63f30e5d-4fa8-5c19-946f-1a524b8b74c1</t>
+          <t>f1106c8b-997a-5d06-a1b6-b30fd8b10523</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Language Coaching Service Variation 6</t>
+          <t>Language &amp; Communication Service Variation 1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -872,11 +872,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Language Coaching</t>
+          <t>Language &amp; Communication</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1700</v>
+        <v>650</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -885,34 +885,34 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
+          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[{"text": "Expert language coaching tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Language Coaching Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.059934+00:00</t>
+          <t>2026-09-05T15:22:47.089751+00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.059934+00:00</t>
+          <t>2026-09-05T15:40:26.060681+00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>f1106c8b-997a-5d06-a1b6-b30fd8b10523</t>
+          <t>d11d4e8e-10ab-52fa-8b31-c974ba7f8906</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Language &amp; Communication Service Variation 1</t>
+          <t>Language &amp; Communication Service Variation 2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -945,24 +945,24 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.089751+00:00</t>
+          <t>2026-09-05T15:22:47.092066+00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.060681+00:00</t>
+          <t>2026-09-05T15:40:26.063121+00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d11d4e8e-10ab-52fa-8b31-c974ba7f8906</t>
+          <t>245d6207-15de-5adc-9b1b-7c387c372955</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Language &amp; Communication Service Variation 2</t>
+          <t>Language &amp; Communication Service Variation 3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>800</v>
+        <v>950</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -995,24 +995,24 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.092066+00:00</t>
+          <t>2026-09-05T15:22:47.094264+00:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.063121+00:00</t>
+          <t>2026-09-05T15:40:26.065533+00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>245d6207-15de-5adc-9b1b-7c387c372955</t>
+          <t>e4f0a121-e2bb-5118-a516-7a3c16944184</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Language &amp; Communication Service Variation 3</t>
+          <t>Language &amp; Communication Service Variation 4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>950</v>
+        <v>1100</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1045,24 +1045,24 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.094264+00:00</t>
+          <t>2026-09-05T15:22:47.096490+00:00</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.065533+00:00</t>
+          <t>2026-09-05T15:40:26.068388+00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>e4f0a121-e2bb-5118-a516-7a3c16944184</t>
+          <t>a05334fd-3b60-510c-ae8c-8d53275a302e</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Language &amp; Communication Service Variation 4</t>
+          <t>Language &amp; Communication Service Variation 5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1100</v>
+        <v>1250</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1095,24 +1095,24 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.096490+00:00</t>
+          <t>2026-09-05T15:22:47.098887+00:00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.068388+00:00</t>
+          <t>2026-09-05T15:40:26.070890+00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>a05334fd-3b60-510c-ae8c-8d53275a302e</t>
+          <t>6cdfea65-f777-5015-ab14-9629e747eb08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Language &amp; Communication Service Variation 5</t>
+          <t>Music &amp; Arts Lessons Service Variation 1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1122,11 +1122,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Language &amp; Communication</t>
+          <t>Music &amp; Arts Lessons</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1250</v>
+        <v>650</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1140,29 +1140,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[{"text": "Professional language &amp; communication coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Language &amp; Communication instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.098887+00:00</t>
+          <t>2026-09-05T15:22:47.046691+00:00</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.070890+00:00</t>
+          <t>2026-09-05T15:40:26.073488+00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6cdfea65-f777-5015-ab14-9629e747eb08</t>
+          <t>41f10521-548d-5a2d-a4a9-840503b42220</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons Service Variation 1</t>
+          <t>Music &amp; Arts Lessons Service Variation 2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1195,24 +1195,24 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.046691+00:00</t>
+          <t>2026-09-05T15:22:47.049835+00:00</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.073488+00:00</t>
+          <t>2026-09-05T15:40:26.076124+00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>41f10521-548d-5a2d-a4a9-840503b42220</t>
+          <t>3c7771ad-a2b2-51ce-8846-bbe481a7c7c1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons Service Variation 2</t>
+          <t>Music &amp; Arts Lessons Service Variation 3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1226,7 +1226,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>800</v>
+        <v>950</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1245,24 +1245,24 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.049835+00:00</t>
+          <t>2026-09-05T15:22:47.052666+00:00</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.076124+00:00</t>
+          <t>2026-09-05T15:40:26.078483+00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3c7771ad-a2b2-51ce-8846-bbe481a7c7c1</t>
+          <t>453266d6-b237-5e06-8df4-33eda2c614ee</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons Service Variation 3</t>
+          <t>Music &amp; Arts Lessons Service Variation 4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>950</v>
+        <v>1100</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1295,24 +1295,24 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.052666+00:00</t>
+          <t>2026-09-05T15:22:47.055059+00:00</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.078483+00:00</t>
+          <t>2026-09-05T15:40:26.081162+00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>453266d6-b237-5e06-8df4-33eda2c614ee</t>
+          <t>479f80e0-44a1-531c-9ad2-ade93e865775</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons Service Variation 4</t>
+          <t>Music &amp; Arts Lessons Service Variation 5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1100</v>
+        <v>1250</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1345,24 +1345,24 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.055059+00:00</t>
+          <t>2026-09-05T15:22:47.057378+00:00</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.081162+00:00</t>
+          <t>2026-09-05T15:40:26.083919+00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>479f80e0-44a1-531c-9ad2-ade93e865775</t>
+          <t>d9cc76c1-de06-5737-8945-30bb558d5a13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons Service Variation 5</t>
+          <t>School Tutoring (K-12) Service Variation 1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1372,11 +1372,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Music &amp; Arts Lessons</t>
+          <t>School Tutoring (K-12)</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1250</v>
+        <v>650</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1390,29 +1390,29 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>[{"text": "Professional music &amp; arts lessons coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Music &amp; Arts Lessons instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.057378+00:00</t>
+          <t>2026-09-05T15:22:47.023255+00:00</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.083919+00:00</t>
+          <t>2026-09-05T15:40:26.087401+00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>d9cc76c1-de06-5737-8945-30bb558d5a13</t>
+          <t>293ae0d9-5f80-5635-93cb-459e7ffcb6c1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 1</t>
+          <t>School Tutoring (K-12) Service Variation 2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1445,24 +1445,24 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.023255+00:00</t>
+          <t>2026-09-05T15:22:47.028305+00:00</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.087401+00:00</t>
+          <t>2026-09-05T15:40:26.089859+00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>293ae0d9-5f80-5635-93cb-459e7ffcb6c1</t>
+          <t>946f1a7c-5278-5372-9aee-571229c7d7a7</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 2</t>
+          <t>School Tutoring (K-12) Service Variation 3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>800</v>
+        <v>950</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1495,24 +1495,24 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.028305+00:00</t>
+          <t>2026-09-05T15:22:47.031218+00:00</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.089859+00:00</t>
+          <t>2026-09-05T15:40:26.092758+00:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>946f1a7c-5278-5372-9aee-571229c7d7a7</t>
+          <t>bf24b529-26a3-56e7-ba4f-85893181cd5d</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 3</t>
+          <t>School Tutoring (K-12) Service Variation 4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>950</v>
+        <v>1100</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1545,24 +1545,24 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.031218+00:00</t>
+          <t>2026-09-05T15:22:47.035452+00:00</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.092758+00:00</t>
+          <t>2026-09-05T15:40:26.095081+00:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>bf24b529-26a3-56e7-ba4f-85893181cd5d</t>
+          <t>e3a74561-e859-5f36-ab07-545c6823fbd1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 4</t>
+          <t>School Tutoring (K-12) Service Variation 5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1576,7 +1576,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1100</v>
+        <v>1250</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1595,24 +1595,24 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.035452+00:00</t>
+          <t>2026-09-05T15:22:47.039114+00:00</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.095081+00:00</t>
+          <t>2026-09-05T15:40:26.098037+00:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>e3a74561-e859-5f36-ab07-545c6823fbd1</t>
+          <t>c9b53453-8a57-5ae6-843c-15688915434b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 5</t>
+          <t>School Tutoring (K-12) Service Variation 6</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1250</v>
+        <v>1400</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1645,24 +1645,24 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.039114+00:00</t>
+          <t>2026-09-05T15:22:47.041425+00:00</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.098037+00:00</t>
+          <t>2026-09-05T15:40:26.101192+00:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>c9b53453-8a57-5ae6-843c-15688915434b</t>
+          <t>d62dfd9c-d29f-576c-9470-2bbae0544e3a</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 6</t>
+          <t>School Tutoring (K-12) Service Variation 7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1676,7 +1676,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1400</v>
+        <v>1550</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1695,24 +1695,24 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.041425+00:00</t>
+          <t>2026-09-05T15:22:47.044343+00:00</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.101192+00:00</t>
+          <t>2026-09-05T15:40:26.103546+00:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>d62dfd9c-d29f-576c-9470-2bbae0544e3a</t>
+          <t>b3caa66a-909e-5c9b-8e28-066ea5298ca7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12) Service Variation 7</t>
+          <t>Skills &amp; Hobby Classes Service Variation 1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1722,11 +1722,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>School Tutoring (K-12)</t>
+          <t>Skills &amp; Hobby Classes</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1550</v>
+        <v>650</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1740,29 +1740,29 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>[{"text": "Professional school tutoring (k-12) coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert School Tutoring (K-12) instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.044343+00:00</t>
+          <t>2026-09-05T15:22:47.077035+00:00</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.103546+00:00</t>
+          <t>2026-09-05T15:40:26.105860+00:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>b3caa66a-909e-5c9b-8e28-066ea5298ca7</t>
+          <t>3a2c9ca8-d9fb-5031-b211-e6031179640d</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Skills &amp; Hobby Classes Service Variation 1</t>
+          <t>Skills &amp; Hobby Classes Service Variation 2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1795,24 +1795,24 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.077035+00:00</t>
+          <t>2026-09-05T15:22:47.079289+00:00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.105860+00:00</t>
+          <t>2026-09-05T15:40:26.108502+00:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3a2c9ca8-d9fb-5031-b211-e6031179640d</t>
+          <t>fd8b9cf7-cd66-5e92-9e64-185217363d64</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Skills &amp; Hobby Classes Service Variation 2</t>
+          <t>Skills &amp; Hobby Classes Service Variation 3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>800</v>
+        <v>950</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1845,24 +1845,24 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.079289+00:00</t>
+          <t>2026-09-05T15:22:47.082206+00:00</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.108502+00:00</t>
+          <t>2026-09-05T15:40:26.110846+00:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>fd8b9cf7-cd66-5e92-9e64-185217363d64</t>
+          <t>df4be4ea-2f76-566a-8ad7-db35cbbfafb0</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Skills &amp; Hobby Classes Service Variation 3</t>
+          <t>Skills &amp; Hobby Classes Service Variation 4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>950</v>
+        <v>1100</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1895,24 +1895,24 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.082206+00:00</t>
+          <t>2026-09-05T15:22:47.085005+00:00</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.110846+00:00</t>
+          <t>2026-09-05T15:40:26.114213+00:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>df4be4ea-2f76-566a-8ad7-db35cbbfafb0</t>
+          <t>22edd7f9-7d44-5119-aacc-7979474a88f5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Skills &amp; Hobby Classes Service Variation 4</t>
+          <t>Skills &amp; Hobby Classes Service Variation 5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1100</v>
+        <v>1250</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1945,24 +1945,24 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.085005+00:00</t>
+          <t>2026-09-05T15:22:47.087244+00:00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.114213+00:00</t>
+          <t>2026-09-05T15:40:26.117877+00:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>22edd7f9-7d44-5119-aacc-7979474a88f5</t>
+          <t>f1093f34-1774-5635-ad64-bb37eb928fb5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Skills &amp; Hobby Classes Service Variation 5</t>
+          <t>Skills &amp; Hobby Classes Service Variation 6</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1250</v>
+        <v>1400</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1995,112 +1995,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-05T15:22:47.087244+00:00</t>
+          <t>2026-09-05T15:40:26.120455+00:00</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:26.117877+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>f1093f34-1774-5635-ad64-bb37eb928fb5</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Skills &amp; Hobby Classes Service Variation 6</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>8. Education, Teachers &amp; Coaching</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Skills &amp; Hobby Classes</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>["Personalised lesson plan preparation", "One-on-one or small group sessions", "Study material and notes", "Progress tracking and feedback reports"]</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>[{"text": "Professional skills &amp; hobby classes coaching tailored to individual learning needs.", "type": "description"}, {"type": "highlights", "items": ["Expert Skills &amp; Hobby Classes instructor", "Customised lesson plans", "Flexible scheduling (online &amp; in-home)", "Regular progress reports"]}, {"type": "excluded_scope", "items": ["Cost of textbooks or printed materials", "Examination registration fees"]}, {"type": "process_steps", "steps": [{"title": "Initial Assessment", "description": "Evaluating the student's current level and learning goals", "step_number": 1}, {"title": "Lesson Planning", "description": "Customising a structured study plan", "step_number": 2}, {"title": "Teaching Sessions", "description": "Conducting focused, interactive lessons", "step_number": 3}, {"title": "Practice &amp; Assignments", "description": "Providing exercises to reinforce concepts", "step_number": 4}, {"title": "Review &amp; Feedback", "description": "Reviewing progress and adjusting the plan as needed", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework before the next session", "Review notes within 24 hours of each session"]}, {"type": "tools_materials", "tools": ["Whiteboard or digital board", "Reference textbooks", "Practice worksheets", "Online resources"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet study environment", "Have necessary stationery and books ready", "Share syllabus or exam board details upfront"]}, {"type": "expected_results", "items": "Measurable improvement in understanding, grades, and confidence."}, {"type": "important_notes", "items": "Minimum 4-session commitment recommended for meaningful progress."}, {"type": "warranty", "details": "Free rescheduling if tutor cancels; satisfaction guarantee on first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "Yes, you can browse tutor profiles and select based on expertise and availability.", "question": "Can I choose the tutor?"}, {"answer": "Yes, all tutoring services are available both online and in-home.", "question": "Are online sessions available?"}, {"answer": "You can request a replacement tutor at no extra cost within the first session.", "question": "What if I want to switch tutors?"}, {"answer": "Yes, we have specialised tutors for JEE, NEET, UPSC, CAT, and other exams.", "question": "Do you cater to competitive exam preparation?"}]}, {"type": "tips", "items": ["Revise notes within 24 hours to retain 80% more."]}, {"dos": ["Attend every session punctually."], "type": "dos_donts", "donts": ["Do not skip assigned practice work between sessions."]}, {"type": "duration", "minutes": 60}]</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
           <t>2026-09-05T15:40:26.120455+00:00</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>2026-09-05T15:40:26.120455+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>1b791937-c35c-5f48-83c8-e2f133823421</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Test Preparation Service Variation 6</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>8. Education, Teachers &amp; Coaching</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Test Preparation</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>["Initial skill assessment", "Personalized lesson plan", "Interactive sessions", "Progress tracking"]</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>[{"text": "Expert test preparation tailored for your specific learning goals.", "type": "description"}, {"type": "highlights", "items": ["Experienced Test Preparation Instructor", "Personalized attention", "Flexible scheduling", "Progress monitoring"]}, {"type": "excluded_scope", "items": ["Cost of specialized learning materials", "Transportation costs (for offline sessions)"]}, {"type": "process_steps", "steps": [{"title": "Assessment", "description": "Evaluating the student's current proficiency level", "step_number": 1}, {"title": "Goal Setting", "description": "Defining clear learning objectives", "step_number": 2}, {"title": "Instruction", "description": "Conducting interactive coaching sessions", "step_number": 3}, {"title": "Practice", "description": "Assigning exercises to reinforce learning", "step_number": 4}, {"title": "Review", "description": "Tracking progress and adjusting the lesson plan", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Complete assigned homework/practice routines", "Review feedback provided by the coach"]}, {"type": "tools_materials", "tools": ["Notebooks/Digital tablets", "Course material/Syllabus", "Subject-specific tools"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure a quiet learning environment", "Provide stable internet for online sessions"]}, {"type": "expected_results", "items": "Noticeable improvement in skills and knowledge."}, {"type": "important_notes", "items": "Consistent attendance is required for best results."}, {"type": "warranty", "details": "Satisfaction guarantee for the first session.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "We offer both online and offline options depending on the service.", "question": "Are the classes online or offline?"}, {"answer": "Basic materials are included; specialized textbooks must be purchased separately.", "question": "Are learning materials provided?"}, {"answer": "We conduct periodic tests and provide detailed progress reports.", "question": "How do you track progress?"}, {"answer": "Yes, sessions can be rescheduled with 24 hours prior notice.", "question": "Can I reschedule a session?"}]}, {"type": "tips", "items": ["Set aside dedicated time for self-study to reinforce class learning."]}, {"dos": ["Participate actively during sessions.", "Ask questions whenever in doubt."], "type": "dos_donts", "donts": ["Do not skip practice assignments."]}, {"type": "duration", "minutes": 60}]</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-09-05T15:22:47.101322+00:00</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>2026-09-05T15:22:47.101322+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>